<commit_message>
Clean manual import fixture emails
</commit_message>
<xml_diff>
--- a/test_uploads/importacao_guiada/alunos_multiplas_abas.xlsx
+++ b/test_uploads/importacao_guiada/alunos_multiplas_abas.xlsx
@@ -497,7 +497,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ana.lima@example.com</t>
+          <t>login-a001@escola.test</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>bruno.reis@example.com</t>
+          <t>portal-8802@escola.test</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -539,11 +539,7 @@
           <t>Carla Dias</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>carla.dias@example.com</t>
-        </is>
-      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>C003</t>
@@ -551,7 +547,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>linha limpa</t>
+          <t>sem email</t>
         </is>
       </c>
     </row>

</xml_diff>